<commit_message>
Apply the doctor's glossary corrections: SWE wording and 'imaging'
- shear wave elastography / SWE -> 'to‘lqin siljish elastografiyasi (SWE)'
- new term 'imaging' -> 'tasvir'
Counts are now 228 = 171 approved + 56 corrected + 1 new.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TpdXy8usyRzAsJppPfUV6H
</commit_message>
<xml_diff>
--- a/docs/glossary/UZI_atamalari_tekshirilgan.xlsx
+++ b/docs/glossary/UZI_atamalari_tekshirilgan.xlsx
@@ -514,6 +514,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="35.05" customHeight="1" s="13">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -526,6 +527,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="13">
       <c r="A5" s="17" t="inlineStr">
         <is>
@@ -598,6 +600,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="13">
       <c r="A12" s="15" t="inlineStr">
         <is>
@@ -714,6 +717,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="13">
       <c r="A23" s="15" t="inlineStr">
         <is>
@@ -729,7 +733,7 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="13">
@@ -739,7 +743,7 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="13">
@@ -749,7 +753,7 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="13">
@@ -769,7 +773,7 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="13">
@@ -782,13 +786,14 @@
         <v>0</v>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>Tekshiruv natijasi</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>Barcha 227 mavjud atama ko‘rib chiqildi; 55 ta atamada tarjima yoki tibbiy izoh aniqlashtirildi.</t>
         </is>
@@ -807,7 +812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J228"/>
+  <dimension ref="A1:J229"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -3550,7 +3555,7 @@
       </c>
       <c r="H64" s="24" t="inlineStr">
         <is>
-          <t>siljish to‘lqini elastografiyasi (SWE)</t>
+          <t>to‘lqin siljish elastografiyasi (SWE)</t>
         </is>
       </c>
       <c r="I64" s="24" t="inlineStr">
@@ -3587,10 +3592,14 @@
       <c r="F65" s="23" t="n"/>
       <c r="G65" s="24" t="inlineStr">
         <is>
-          <t>To'g'ri</t>
-        </is>
-      </c>
-      <c r="H65" s="24" t="n"/>
+          <t>Tuzatildi</t>
+        </is>
+      </c>
+      <c r="H65" s="24" t="inlineStr">
+        <is>
+          <t>to‘lqin siljish elastografiyasi (SWE)</t>
+        </is>
+      </c>
       <c r="I65" s="24" t="n"/>
       <c r="J65" s="24" t="inlineStr">
         <is>
@@ -9975,6 +9984,44 @@
       <c r="H228" s="24" t="n"/>
       <c r="I228" s="24" t="n"/>
       <c r="J228" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="22" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" s="23" t="inlineStr">
+        <is>
+          <t>Tasvir va exogenlik</t>
+        </is>
+      </c>
+      <c r="C229" s="23" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="D229" s="23" t="n"/>
+      <c r="E229" s="23" t="inlineStr">
+        <is>
+          <t>tasvir</t>
+        </is>
+      </c>
+      <c r="F229" s="23" t="inlineStr">
+        <is>
+          <t>Ultratovush yordamida olingan tasvir yoki tasvir olish jarayoni (masalan, "elastography imaging" — elastografiya tasviri).</t>
+        </is>
+      </c>
+      <c r="G229" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H229" s="24" t="n"/>
+      <c r="I229" s="24" t="n"/>
+      <c r="J229" s="24" t="inlineStr">
         <is>
           <t>Yo'q</t>
         </is>

</xml_diff>

<commit_message>
UZI glossary: 16 terms from the translator skill; the doctor's translation decisions
The doctor approved (2026-10-18) adding the medical-uzbek-translator skill's draft terms: 16 were new
(229-244: pancreatitis types, peripancreatic fluid, fluid collection, omental bursa, atrophic, pseudocyst,
pseudoaneurysm, splenic artery and window, cross and long section, vascularity, epigastric pain, upper
limit of normal, caudally); 9 were already in the glossary. calcification stays 'kalsifikat', centimetres
stay 'cm'. The translation standard records the decisions; the 12 doubtful entries went to the doctor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCMr8axiH8WW9Y4zGdu8Lo
</commit_message>
<xml_diff>
--- a/docs/glossary/UZI_atamalari_tekshirilgan.xlsx
+++ b/docs/glossary/UZI_atamalari_tekshirilgan.xlsx
@@ -514,7 +514,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="35.05" customHeight="1" s="13">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -527,7 +526,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="13">
       <c r="A5" s="17" t="inlineStr">
         <is>
@@ -600,7 +598,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="13">
       <c r="A12" s="15" t="inlineStr">
         <is>
@@ -717,7 +714,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="13">
       <c r="A23" s="15" t="inlineStr">
         <is>
@@ -786,7 +782,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
@@ -812,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J229"/>
+  <dimension ref="A1:J245"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -10022,6 +10017,582 @@
       <c r="H229" s="24" t="n"/>
       <c r="I229" s="24" t="n"/>
       <c r="J229" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="22" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" s="23" t="inlineStr">
+        <is>
+          <t>Qorin bo'shlig'i a'zolari</t>
+        </is>
+      </c>
+      <c r="C230" s="23" t="inlineStr">
+        <is>
+          <t>interstitial edematous pancreatitis</t>
+        </is>
+      </c>
+      <c r="D230" s="23" t="inlineStr">
+        <is>
+          <t>interstitial oedematous pancreatitis; edematous pancreatitis</t>
+        </is>
+      </c>
+      <c r="E230" s="23" t="inlineStr">
+        <is>
+          <t>interstitsial (shishli) pankreatit</t>
+        </is>
+      </c>
+      <c r="F230" s="23" t="n"/>
+      <c r="G230" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H230" s="24" t="n"/>
+      <c r="I230" s="24" t="n"/>
+      <c r="J230" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="22" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" s="23" t="inlineStr">
+        <is>
+          <t>Qorin bo'shlig'i a'zolari</t>
+        </is>
+      </c>
+      <c r="C231" s="23" t="inlineStr">
+        <is>
+          <t>necrotizing pancreatitis</t>
+        </is>
+      </c>
+      <c r="D231" s="23" t="inlineStr">
+        <is>
+          <t>necrotising pancreatitis</t>
+        </is>
+      </c>
+      <c r="E231" s="23" t="inlineStr">
+        <is>
+          <t>nekrotik pankreatit</t>
+        </is>
+      </c>
+      <c r="F231" s="23" t="n"/>
+      <c r="G231" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H231" s="24" t="n"/>
+      <c r="I231" s="24" t="n"/>
+      <c r="J231" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="22" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" s="23" t="inlineStr">
+        <is>
+          <t>Qorin bo'shlig'i a'zolari</t>
+        </is>
+      </c>
+      <c r="C232" s="23" t="inlineStr">
+        <is>
+          <t>peripancreatic fluid</t>
+        </is>
+      </c>
+      <c r="D232" s="23" t="n"/>
+      <c r="E232" s="23" t="inlineStr">
+        <is>
+          <t>bez atrofidagi suyuqlik</t>
+        </is>
+      </c>
+      <c r="F232" s="23" t="n"/>
+      <c r="G232" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H232" s="24" t="n"/>
+      <c r="I232" s="24" t="n"/>
+      <c r="J232" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="22" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" s="23" t="inlineStr">
+        <is>
+          <t>Umumiy patologiya</t>
+        </is>
+      </c>
+      <c r="C233" s="23" t="inlineStr">
+        <is>
+          <t>fluid collection</t>
+        </is>
+      </c>
+      <c r="D233" s="23" t="n"/>
+      <c r="E233" s="23" t="inlineStr">
+        <is>
+          <t>suyuqlik to'plami</t>
+        </is>
+      </c>
+      <c r="F233" s="23" t="n"/>
+      <c r="G233" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H233" s="24" t="n"/>
+      <c r="I233" s="24" t="n"/>
+      <c r="J233" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="22" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" s="23" t="inlineStr">
+        <is>
+          <t>Qorin bo'shlig'i a'zolari</t>
+        </is>
+      </c>
+      <c r="C234" s="23" t="inlineStr">
+        <is>
+          <t>omental bursa</t>
+        </is>
+      </c>
+      <c r="D234" s="23" t="inlineStr">
+        <is>
+          <t>lesser sac</t>
+        </is>
+      </c>
+      <c r="E234" s="23" t="inlineStr">
+        <is>
+          <t>charvi xaltasi (omental bursa)</t>
+        </is>
+      </c>
+      <c r="F234" s="23" t="n"/>
+      <c r="G234" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H234" s="24" t="n"/>
+      <c r="I234" s="24" t="n"/>
+      <c r="J234" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="22" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" s="23" t="inlineStr">
+        <is>
+          <t>Umumiy patologiya</t>
+        </is>
+      </c>
+      <c r="C235" s="23" t="inlineStr">
+        <is>
+          <t>atrophic</t>
+        </is>
+      </c>
+      <c r="D235" s="23" t="n"/>
+      <c r="E235" s="23" t="inlineStr">
+        <is>
+          <t>atrofik</t>
+        </is>
+      </c>
+      <c r="F235" s="23" t="n"/>
+      <c r="G235" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H235" s="24" t="n"/>
+      <c r="I235" s="24" t="n"/>
+      <c r="J235" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="22" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" s="23" t="inlineStr">
+        <is>
+          <t>Umumiy patologiya</t>
+        </is>
+      </c>
+      <c r="C236" s="23" t="inlineStr">
+        <is>
+          <t>pseudocyst</t>
+        </is>
+      </c>
+      <c r="D236" s="23" t="n"/>
+      <c r="E236" s="23" t="inlineStr">
+        <is>
+          <t>psevdokista</t>
+        </is>
+      </c>
+      <c r="F236" s="23" t="n"/>
+      <c r="G236" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H236" s="24" t="n"/>
+      <c r="I236" s="24" t="n"/>
+      <c r="J236" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="22" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" s="23" t="inlineStr">
+        <is>
+          <t>Umumiy patologiya</t>
+        </is>
+      </c>
+      <c r="C237" s="23" t="inlineStr">
+        <is>
+          <t>pseudoaneurysm</t>
+        </is>
+      </c>
+      <c r="D237" s="23" t="inlineStr">
+        <is>
+          <t>false aneurysm</t>
+        </is>
+      </c>
+      <c r="E237" s="23" t="inlineStr">
+        <is>
+          <t>psevdoanevrizma</t>
+        </is>
+      </c>
+      <c r="F237" s="23" t="n"/>
+      <c r="G237" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H237" s="24" t="n"/>
+      <c r="I237" s="24" t="n"/>
+      <c r="J237" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="22" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" s="23" t="inlineStr">
+        <is>
+          <t>Doppler</t>
+        </is>
+      </c>
+      <c r="C238" s="23" t="inlineStr">
+        <is>
+          <t>splenic artery</t>
+        </is>
+      </c>
+      <c r="D238" s="23" t="n"/>
+      <c r="E238" s="23" t="inlineStr">
+        <is>
+          <t>taloq arteriyasi</t>
+        </is>
+      </c>
+      <c r="F238" s="23" t="n"/>
+      <c r="G238" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H238" s="24" t="n"/>
+      <c r="I238" s="24" t="n"/>
+      <c r="J238" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="22" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" s="23" t="inlineStr">
+        <is>
+          <t>Tasvir va exogenlik</t>
+        </is>
+      </c>
+      <c r="C239" s="23" t="inlineStr">
+        <is>
+          <t>splenic window</t>
+        </is>
+      </c>
+      <c r="D239" s="23" t="n"/>
+      <c r="E239" s="23" t="inlineStr">
+        <is>
+          <t>taloq oynasi (taloq orqali kirish)</t>
+        </is>
+      </c>
+      <c r="F239" s="23" t="n"/>
+      <c r="G239" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H239" s="24" t="n"/>
+      <c r="I239" s="24" t="n"/>
+      <c r="J239" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="22" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" s="23" t="inlineStr">
+        <is>
+          <t>Tasvir va exogenlik</t>
+        </is>
+      </c>
+      <c r="C240" s="23" t="inlineStr">
+        <is>
+          <t>cross section</t>
+        </is>
+      </c>
+      <c r="D240" s="23" t="inlineStr">
+        <is>
+          <t>cross-section; transverse section</t>
+        </is>
+      </c>
+      <c r="E240" s="23" t="inlineStr">
+        <is>
+          <t>ko'ndalang kesim</t>
+        </is>
+      </c>
+      <c r="F240" s="23" t="n"/>
+      <c r="G240" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H240" s="24" t="n"/>
+      <c r="I240" s="24" t="n"/>
+      <c r="J240" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="22" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" s="23" t="inlineStr">
+        <is>
+          <t>Tasvir va exogenlik</t>
+        </is>
+      </c>
+      <c r="C241" s="23" t="inlineStr">
+        <is>
+          <t>long section</t>
+        </is>
+      </c>
+      <c r="D241" s="23" t="inlineStr">
+        <is>
+          <t>longitudinal section</t>
+        </is>
+      </c>
+      <c r="E241" s="23" t="inlineStr">
+        <is>
+          <t>bo'ylama kesim</t>
+        </is>
+      </c>
+      <c r="F241" s="23" t="n"/>
+      <c r="G241" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H241" s="24" t="n"/>
+      <c r="I241" s="24" t="n"/>
+      <c r="J241" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="22" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" s="23" t="inlineStr">
+        <is>
+          <t>Doppler</t>
+        </is>
+      </c>
+      <c r="C242" s="23" t="inlineStr">
+        <is>
+          <t>vascularity</t>
+        </is>
+      </c>
+      <c r="D242" s="23" t="inlineStr">
+        <is>
+          <t>vascularization; vascularisation</t>
+        </is>
+      </c>
+      <c r="E242" s="23" t="inlineStr">
+        <is>
+          <t>qon bilan ta'minlanish (vaskulyarizatsiya)</t>
+        </is>
+      </c>
+      <c r="F242" s="23" t="n"/>
+      <c r="G242" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H242" s="24" t="n"/>
+      <c r="I242" s="24" t="n"/>
+      <c r="J242" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="22" t="n">
+        <v>242</v>
+      </c>
+      <c r="B243" s="23" t="inlineStr">
+        <is>
+          <t>Umumiy patologiya</t>
+        </is>
+      </c>
+      <c r="C243" s="23" t="inlineStr">
+        <is>
+          <t>epigastric pain</t>
+        </is>
+      </c>
+      <c r="D243" s="23" t="n"/>
+      <c r="E243" s="23" t="inlineStr">
+        <is>
+          <t>epigastral og'riq</t>
+        </is>
+      </c>
+      <c r="F243" s="23" t="n"/>
+      <c r="G243" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H243" s="24" t="n"/>
+      <c r="I243" s="24" t="n"/>
+      <c r="J243" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="22" t="n">
+        <v>243</v>
+      </c>
+      <c r="B244" s="23" t="inlineStr">
+        <is>
+          <t>Umumiy patologiya</t>
+        </is>
+      </c>
+      <c r="C244" s="23" t="inlineStr">
+        <is>
+          <t>upper limit of normal</t>
+        </is>
+      </c>
+      <c r="D244" s="23" t="inlineStr">
+        <is>
+          <t>ULN</t>
+        </is>
+      </c>
+      <c r="E244" s="23" t="inlineStr">
+        <is>
+          <t>normaning yuqori chegarasi</t>
+        </is>
+      </c>
+      <c r="F244" s="23" t="n"/>
+      <c r="G244" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H244" s="24" t="n"/>
+      <c r="I244" s="24" t="n"/>
+      <c r="J244" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="22" t="n">
+        <v>244</v>
+      </c>
+      <c r="B245" s="23" t="inlineStr">
+        <is>
+          <t>Tasvir va exogenlik</t>
+        </is>
+      </c>
+      <c r="C245" s="23" t="inlineStr">
+        <is>
+          <t>caudally</t>
+        </is>
+      </c>
+      <c r="D245" s="23" t="n"/>
+      <c r="E245" s="23" t="inlineStr">
+        <is>
+          <t>kaudal yo'nalishda (pastga qarab)</t>
+        </is>
+      </c>
+      <c r="F245" s="23" t="n"/>
+      <c r="G245" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H245" s="24" t="n"/>
+      <c r="I245" s="24" t="n"/>
+      <c r="J245" s="24" t="inlineStr">
         <is>
           <t>Yo'q</t>
         </is>

</xml_diff>

<commit_message>
SHOKALON translation QA: notes in SRT, untranslated and repeated cues; batch packer
- check_translation.py: an error for review marks or notes inside the subtitle
  text and for cues left in English; a warning for a cue repeating the previous
  translation.
- package_translations.py checks a batch (section or chapter) against the
  originals, zips only error-free files under their SHOKALON names and writes
  HISOBOT.md: counts, errors, untranslated files, warnings, translator notes.
- Glossary 269: lymphatic vessel = limfa tomiri (doctor's requirement).
- The translation standard records the doctor's 2026-10-18 requirements.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JkhWytwk2bETHyYPZ9J87d
</commit_message>
<xml_diff>
--- a/docs/glossary/UZI_atamalari_tekshirilgan.xlsx
+++ b/docs/glossary/UZI_atamalari_tekshirilgan.xlsx
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J269"/>
+  <dimension ref="A1:J270"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -11469,6 +11469,44 @@
       <c r="H269" s="24" t="n"/>
       <c r="I269" s="24" t="n"/>
       <c r="J269" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="22" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" s="23" t="inlineStr">
+        <is>
+          <t>Qorin bo'shlig'i a'zolari</t>
+        </is>
+      </c>
+      <c r="C270" s="23" t="inlineStr">
+        <is>
+          <t>lymphatic vessel</t>
+        </is>
+      </c>
+      <c r="D270" s="23" t="inlineStr">
+        <is>
+          <t>lymphatic vessels; lymph vessel; lymph vessels</t>
+        </is>
+      </c>
+      <c r="E270" s="23" t="inlineStr">
+        <is>
+          <t>limfa tomiri</t>
+        </is>
+      </c>
+      <c r="F270" s="23" t="n"/>
+      <c r="G270" s="24" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="H270" s="24" t="n"/>
+      <c r="I270" s="24" t="n"/>
+      <c r="J270" s="24" t="inlineStr">
         <is>
           <t>Yo'q</t>
         </is>

</xml_diff>

<commit_message>
Glossary: plane is kesim (scanning plane), never samolyot
The lessons translated "plane" both as kesim and as samolyot (aircraft). The
reviewed glossary gets plane, sagittal, transverse and coronal plane, so new
translations and Claude's checks use kesim.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JkhWytwk2bETHyYPZ9J87d
</commit_message>
<xml_diff>
--- a/docs/glossary/UZI_atamalari_tekshirilgan.xlsx
+++ b/docs/glossary/UZI_atamalari_tekshirilgan.xlsx
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J270"/>
+  <dimension ref="A1:J274"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -11507,6 +11507,151 @@
       <c r="H270" s="24" t="n"/>
       <c r="I270" s="24" t="n"/>
       <c r="J270" s="24" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Tasvir va exogenlik</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>plane</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>planes; scan plane; scanning plane; imaging plane; image plane; section plane</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>kesim (tekislik)</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Ultratovush kesimi (skanerlash tekisligi). 'Samolyot' deb tarjima qilinmaydi.</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Tasvir va exogenlik</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>sagittal plane</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>sagittal section; sagittal view; sagittal planes</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>sagittal kesim</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Tasvir va exogenlik</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>transverse plane</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>transverse view; axial plane; transverse planes</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>ko‘ndalang kesim</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Tasvir va exogenlik</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>coronal plane</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>coronal section; coronal view; coronal planes</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>frontal (koronar) kesim</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Yangi</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
         <is>
           <t>Yo'q</t>
         </is>

</xml_diff>

<commit_message>
Glossary: coronal plane is koronal kesim
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JkhWytwk2bETHyYPZ9J87d
</commit_message>
<xml_diff>
--- a/docs/glossary/UZI_atamalari_tekshirilgan.xlsx
+++ b/docs/glossary/UZI_atamalari_tekshirilgan.xlsx
@@ -11513,145 +11513,145 @@
       </c>
     </row>
     <row r="271">
-      <c r="A271" t="n">
+      <c r="A271" s="12" t="n">
         <v>270</v>
       </c>
-      <c r="B271" t="inlineStr">
+      <c r="B271" s="12" t="inlineStr">
         <is>
           <t>Tasvir va exogenlik</t>
         </is>
       </c>
-      <c r="C271" t="inlineStr">
+      <c r="C271" s="12" t="inlineStr">
         <is>
           <t>plane</t>
         </is>
       </c>
-      <c r="D271" t="inlineStr">
+      <c r="D271" s="12" t="inlineStr">
         <is>
           <t>planes; scan plane; scanning plane; imaging plane; image plane; section plane</t>
         </is>
       </c>
-      <c r="E271" t="inlineStr">
+      <c r="E271" s="12" t="inlineStr">
         <is>
           <t>kesim (tekislik)</t>
         </is>
       </c>
-      <c r="F271" t="inlineStr">
+      <c r="F271" s="12" t="inlineStr">
         <is>
           <t>Ultratovush kesimi (skanerlash tekisligi). 'Samolyot' deb tarjima qilinmaydi.</t>
         </is>
       </c>
-      <c r="G271" t="inlineStr">
+      <c r="G271" s="12" t="inlineStr">
         <is>
           <t>Yangi</t>
         </is>
       </c>
-      <c r="J271" t="inlineStr">
+      <c r="J271" s="12" t="inlineStr">
         <is>
           <t>Yo'q</t>
         </is>
       </c>
     </row>
     <row r="272">
-      <c r="A272" t="n">
+      <c r="A272" s="12" t="n">
         <v>271</v>
       </c>
-      <c r="B272" t="inlineStr">
+      <c r="B272" s="12" t="inlineStr">
         <is>
           <t>Tasvir va exogenlik</t>
         </is>
       </c>
-      <c r="C272" t="inlineStr">
+      <c r="C272" s="12" t="inlineStr">
         <is>
           <t>sagittal plane</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr">
+      <c r="D272" s="12" t="inlineStr">
         <is>
           <t>sagittal section; sagittal view; sagittal planes</t>
         </is>
       </c>
-      <c r="E272" t="inlineStr">
+      <c r="E272" s="12" t="inlineStr">
         <is>
           <t>sagittal kesim</t>
         </is>
       </c>
-      <c r="G272" t="inlineStr">
+      <c r="G272" s="12" t="inlineStr">
         <is>
           <t>Yangi</t>
         </is>
       </c>
-      <c r="J272" t="inlineStr">
+      <c r="J272" s="12" t="inlineStr">
         <is>
           <t>Yo'q</t>
         </is>
       </c>
     </row>
     <row r="273">
-      <c r="A273" t="n">
+      <c r="A273" s="12" t="n">
         <v>272</v>
       </c>
-      <c r="B273" t="inlineStr">
+      <c r="B273" s="12" t="inlineStr">
         <is>
           <t>Tasvir va exogenlik</t>
         </is>
       </c>
-      <c r="C273" t="inlineStr">
+      <c r="C273" s="12" t="inlineStr">
         <is>
           <t>transverse plane</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr">
+      <c r="D273" s="12" t="inlineStr">
         <is>
           <t>transverse view; axial plane; transverse planes</t>
         </is>
       </c>
-      <c r="E273" t="inlineStr">
+      <c r="E273" s="12" t="inlineStr">
         <is>
           <t>ko‘ndalang kesim</t>
         </is>
       </c>
-      <c r="G273" t="inlineStr">
+      <c r="G273" s="12" t="inlineStr">
         <is>
           <t>Yangi</t>
         </is>
       </c>
-      <c r="J273" t="inlineStr">
+      <c r="J273" s="12" t="inlineStr">
         <is>
           <t>Yo'q</t>
         </is>
       </c>
     </row>
     <row r="274">
-      <c r="A274" t="n">
+      <c r="A274" s="12" t="n">
         <v>273</v>
       </c>
-      <c r="B274" t="inlineStr">
+      <c r="B274" s="12" t="inlineStr">
         <is>
           <t>Tasvir va exogenlik</t>
         </is>
       </c>
-      <c r="C274" t="inlineStr">
+      <c r="C274" s="12" t="inlineStr">
         <is>
           <t>coronal plane</t>
         </is>
       </c>
-      <c r="D274" t="inlineStr">
+      <c r="D274" s="12" t="inlineStr">
         <is>
           <t>coronal section; coronal view; coronal planes</t>
         </is>
       </c>
-      <c r="E274" t="inlineStr">
-        <is>
-          <t>frontal (koronar) kesim</t>
-        </is>
-      </c>
-      <c r="G274" t="inlineStr">
+      <c r="E274" s="12" t="inlineStr">
+        <is>
+          <t>koronal kesim</t>
+        </is>
+      </c>
+      <c r="G274" s="12" t="inlineStr">
         <is>
           <t>Yangi</t>
         </is>
       </c>
-      <c r="J274" t="inlineStr">
+      <c r="J274" s="12" t="inlineStr">
         <is>
           <t>Yo'q</t>
         </is>

</xml_diff>